<commit_message>
task132 figure-neutral cleanup: one PSU serial sequence ahead of the relays, a recorded disposition for every failed module, per-crew wording, Veldtek letterhead and ordering terms, RTU-only rows off the approved sheet, scrapping reasons on the rebuild e-waste orders; no graded figure moved (checks 1,948, verifier green)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task132/target/protection_renewal_program_2026.xlsx
+++ b/task132/target/protection_renewal_program_2026.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Approved 2026'!$A$3:$H$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Approved 2026'!$A$3:$H$150</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2025 plan (superseded)'!$A$3:$H$126</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1661" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="599">
   <si>
     <t>Protection Renewal Program 2026-2035, approved by the Board 19 March 2026 (resolution 2026-07)</t>
   </si>
@@ -1589,10 +1589,202 @@
     <t>Replace feeder relays F01-F32 and RTU, IEC 61850 station bus</t>
   </si>
   <si>
-    <t>DS-028</t>
-  </si>
-  <si>
-    <t>Ostrander</t>
+    <t>DS-037</t>
+  </si>
+  <si>
+    <t>Fontbrune</t>
+  </si>
+  <si>
+    <t>DS-077</t>
+  </si>
+  <si>
+    <t>Tamblyn Line</t>
+  </si>
+  <si>
+    <t>DS-084</t>
+  </si>
+  <si>
+    <t>Dowling Road</t>
+  </si>
+  <si>
+    <t>DS-085</t>
+  </si>
+  <si>
+    <t>Hurlbut</t>
+  </si>
+  <si>
+    <t>DS-092</t>
+  </si>
+  <si>
+    <t>Doupe</t>
+  </si>
+  <si>
+    <t>F05, RTU</t>
+  </si>
+  <si>
+    <t>Replace VPR-220 feeder protection F05 and RTU</t>
+  </si>
+  <si>
+    <t>DS-096</t>
+  </si>
+  <si>
+    <t>Carscadden Road</t>
+  </si>
+  <si>
+    <t>Feeder protection replacement F01-F09, new P&amp;C panels</t>
+  </si>
+  <si>
+    <t>DS-109</t>
+  </si>
+  <si>
+    <t>Torbrae</t>
+  </si>
+  <si>
+    <t>TS-17</t>
+  </si>
+  <si>
+    <t>Wanatami Road</t>
+  </si>
+  <si>
+    <t>Feeder protection and control replacement F01-F27 (VPR-220 feeders F26-F27)</t>
+  </si>
+  <si>
+    <t>Protection Renewal Program, 2025 planning version (superseded by the approved 2026 program)</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F05</t>
+  </si>
+  <si>
+    <t>F01-F31</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F31</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F07</t>
+  </si>
+  <si>
+    <t>F01-F25</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F25</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F25, new panels</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F17</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F05, new panels</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F06</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F08, new panels</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F09, new panels</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F05</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F20</t>
+  </si>
+  <si>
+    <t>P&amp;C rebuild with new control building, feeders F01-F20</t>
+  </si>
+  <si>
+    <t>Feeder protection replacement F01-F17, new P&amp;C panels</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F05</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F09</t>
+  </si>
+  <si>
+    <t>F01-F33</t>
+  </si>
+  <si>
+    <t>Feeder protection and control replacement F01-F33</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F31, new panels</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F06</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F27</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F06, new panels</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F08</t>
+  </si>
+  <si>
+    <t>Replace VPR-340 feeder relays F01-F07</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F08</t>
+  </si>
+  <si>
+    <t>F01-F18</t>
+  </si>
+  <si>
+    <t>Replace feeder relays F01-F18 and RTU, IEC 61850 station bus</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F25</t>
+  </si>
+  <si>
+    <t>F01-F30</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F30, panel rewiring and DC upgrade</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F09</t>
+  </si>
+  <si>
+    <t>F01-F28</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F28</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F22</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F06</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F21</t>
+  </si>
+  <si>
+    <t>Feeder protection replacement F01-F18, new P&amp;C panels</t>
+  </si>
+  <si>
+    <t>VPR-340 feeder protection replacement F01-F32</t>
+  </si>
+  <si>
+    <t>Replace feeder protection F01-F07, new panels</t>
+  </si>
+  <si>
+    <t>Feeder relay replacement F01-F32</t>
+  </si>
+  <si>
+    <t>PRP-204</t>
+  </si>
+  <si>
+    <t>DS-054</t>
+  </si>
+  <si>
+    <t>Côte-Rouge</t>
   </si>
   <si>
     <t>RTU</t>
@@ -1601,210 +1793,6 @@
     <t>RTU replacement and SCADA cutover</t>
   </si>
   <si>
-    <t>DS-037</t>
-  </si>
-  <si>
-    <t>Fontbrune</t>
-  </si>
-  <si>
-    <t>DS-074</t>
-  </si>
-  <si>
-    <t>Craigellan</t>
-  </si>
-  <si>
-    <t>DS-077</t>
-  </si>
-  <si>
-    <t>Tamblyn Line</t>
-  </si>
-  <si>
-    <t>DS-084</t>
-  </si>
-  <si>
-    <t>Dowling Road</t>
-  </si>
-  <si>
-    <t>DS-085</t>
-  </si>
-  <si>
-    <t>Hurlbut</t>
-  </si>
-  <si>
-    <t>DS-092</t>
-  </si>
-  <si>
-    <t>Doupe</t>
-  </si>
-  <si>
-    <t>F05, RTU</t>
-  </si>
-  <si>
-    <t>Replace VPR-220 feeder protection F05 and RTU</t>
-  </si>
-  <si>
-    <t>DS-096</t>
-  </si>
-  <si>
-    <t>Carscadden Road</t>
-  </si>
-  <si>
-    <t>Feeder protection replacement F01-F09, new P&amp;C panels</t>
-  </si>
-  <si>
-    <t>DS-109</t>
-  </si>
-  <si>
-    <t>Torbrae</t>
-  </si>
-  <si>
-    <t>TS-17</t>
-  </si>
-  <si>
-    <t>Wanatami Road</t>
-  </si>
-  <si>
-    <t>Feeder protection and control replacement F01-F27 (VPR-220 feeders F26-F27)</t>
-  </si>
-  <si>
-    <t>Protection Renewal Program, 2025 planning version (superseded by the approved 2026 program)</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F05</t>
-  </si>
-  <si>
-    <t>F01-F31</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F31</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F07</t>
-  </si>
-  <si>
-    <t>F01-F25</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F25</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F25, new panels</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F17</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F05, new panels</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F06</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F08, new panels</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F09, new panels</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F05</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F20</t>
-  </si>
-  <si>
-    <t>P&amp;C rebuild with new control building, feeders F01-F20</t>
-  </si>
-  <si>
-    <t>Feeder protection replacement F01-F17, new P&amp;C panels</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F05</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F09</t>
-  </si>
-  <si>
-    <t>F01-F33</t>
-  </si>
-  <si>
-    <t>Feeder protection and control replacement F01-F33</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F31, new panels</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F06</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F27</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F06, new panels</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F08</t>
-  </si>
-  <si>
-    <t>Replace VPR-340 feeder relays F01-F07</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F08</t>
-  </si>
-  <si>
-    <t>F01-F18</t>
-  </si>
-  <si>
-    <t>Replace feeder relays F01-F18 and RTU, IEC 61850 station bus</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F25</t>
-  </si>
-  <si>
-    <t>F01-F30</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F30, panel rewiring and DC upgrade</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F09</t>
-  </si>
-  <si>
-    <t>F01-F28</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F28</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F22</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F06</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F21</t>
-  </si>
-  <si>
-    <t>Feeder protection replacement F01-F18, new P&amp;C panels</t>
-  </si>
-  <si>
-    <t>VPR-340 feeder protection replacement F01-F32</t>
-  </si>
-  <si>
-    <t>Replace feeder protection F01-F07, new panels</t>
-  </si>
-  <si>
-    <t>Feeder relay replacement F01-F32</t>
-  </si>
-  <si>
-    <t>PRP-204</t>
-  </si>
-  <si>
-    <t>DS-054</t>
-  </si>
-  <si>
-    <t>Côte-Rouge</t>
-  </si>
-  <si>
     <t>Program management notes, P&amp;C Asset Planning. The program is approved by the Board each March with the capital budget; the approved version replaces the planning version of the year before.</t>
   </si>
   <si>
@@ -1823,7 +1811,7 @@
     <t>Bay ranges are copied from the station single-line and take in spare bays and any feeders still on other relay types; the new panels are built for the full range.</t>
   </si>
   <si>
-    <t>Scheme numbers are assigned when a scheme first enters the program and do not change between versions. RTU-only schemes moved to the SCADA upgrade program in 2026 are no longer listed here.</t>
+    <t>Scheme numbers are assigned when a scheme first enters the program and do not change between versions. RTU-only schemes moved to the SCADA upgrade program with the 2026 approval and are no longer listed here; an RTU replaced together with feeder protection stays in that scheme.</t>
   </si>
   <si>
     <t>Stations rebuilt under the 2022-2025 station renewals are complete and are not listed.</t>
@@ -2197,7 +2185,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B686CAD1-F2C9-432F-BAC8-C5EE76427797}">
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -5530,13 +5518,13 @@
         <v>523</v>
       </c>
       <c r="E143" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F143" t="s">
-        <v>524</v>
+        <v>134</v>
       </c>
       <c r="G143" t="s">
-        <v>525</v>
+        <v>245</v>
       </c>
       <c r="H143" s="4" t="s">
         <v>517</v>
@@ -5544,10 +5532,10 @@
     </row>
     <row r="144" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C144" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="D144" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="E144" t="s">
         <v>29</v>
@@ -5564,19 +5552,19 @@
     </row>
     <row r="145" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C145" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D145" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E145" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F145" t="s">
-        <v>524</v>
+        <v>59</v>
       </c>
       <c r="G145" t="s">
-        <v>525</v>
+        <v>60</v>
       </c>
       <c r="H145" s="4" t="s">
         <v>517</v>
@@ -5584,19 +5572,19 @@
     </row>
     <row r="146" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C146" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D146" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="E146" t="s">
         <v>29</v>
       </c>
       <c r="F146" t="s">
-        <v>134</v>
+        <v>59</v>
       </c>
       <c r="G146" t="s">
-        <v>245</v>
+        <v>83</v>
       </c>
       <c r="H146" s="4" t="s">
         <v>517</v>
@@ -5604,19 +5592,19 @@
     </row>
     <row r="147" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C147" t="s">
+        <v>530</v>
+      </c>
+      <c r="D147" t="s">
+        <v>531</v>
+      </c>
+      <c r="E147" t="s">
+        <v>18</v>
+      </c>
+      <c r="F147" t="s">
         <v>532</v>
       </c>
-      <c r="D147" t="s">
+      <c r="G147" t="s">
         <v>533</v>
-      </c>
-      <c r="E147" t="s">
-        <v>29</v>
-      </c>
-      <c r="F147" t="s">
-        <v>59</v>
-      </c>
-      <c r="G147" t="s">
-        <v>60</v>
       </c>
       <c r="H147" s="4" t="s">
         <v>517</v>
@@ -5630,13 +5618,13 @@
         <v>535</v>
       </c>
       <c r="E148" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F148" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G148" t="s">
-        <v>83</v>
+        <v>536</v>
       </c>
       <c r="H148" s="4" t="s">
         <v>517</v>
@@ -5644,19 +5632,19 @@
     </row>
     <row r="149" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C149" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D149" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E149" t="s">
         <v>18</v>
       </c>
       <c r="F149" t="s">
-        <v>538</v>
+        <v>19</v>
       </c>
       <c r="G149" t="s">
-        <v>539</v>
+        <v>68</v>
       </c>
       <c r="H149" s="4" t="s">
         <v>517</v>
@@ -5664,66 +5652,26 @@
     </row>
     <row r="150" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C150" t="s">
+        <v>539</v>
+      </c>
+      <c r="D150" t="s">
         <v>540</v>
       </c>
-      <c r="D150" t="s">
+      <c r="E150" t="s">
+        <v>29</v>
+      </c>
+      <c r="F150" t="s">
+        <v>480</v>
+      </c>
+      <c r="G150" t="s">
         <v>541</v>
-      </c>
-      <c r="E150" t="s">
-        <v>18</v>
-      </c>
-      <c r="F150" t="s">
-        <v>44</v>
-      </c>
-      <c r="G150" t="s">
-        <v>542</v>
       </c>
       <c r="H150" s="4" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="151" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C151" t="s">
-        <v>543</v>
-      </c>
-      <c r="D151" t="s">
-        <v>544</v>
-      </c>
-      <c r="E151" t="s">
-        <v>18</v>
-      </c>
-      <c r="F151" t="s">
-        <v>19</v>
-      </c>
-      <c r="G151" t="s">
-        <v>68</v>
-      </c>
-      <c r="H151" s="4" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="152" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C152" t="s">
-        <v>545</v>
-      </c>
-      <c r="D152" t="s">
-        <v>546</v>
-      </c>
-      <c r="E152" t="s">
-        <v>29</v>
-      </c>
-      <c r="F152" t="s">
-        <v>480</v>
-      </c>
-      <c r="G152" t="s">
-        <v>547</v>
-      </c>
-      <c r="H152" s="4" t="s">
-        <v>517</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:H152"/>
+  <autoFilter ref="A3:H150"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5745,7 +5693,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5814,7 +5762,7 @@
         <v>59</v>
       </c>
       <c r="G5" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="H5" s="3">
         <v>46113</v>
@@ -5834,10 +5782,10 @@
         <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="G6" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="H6" s="3">
         <v>46113</v>
@@ -5906,7 +5854,7 @@
         <v>13</v>
       </c>
       <c r="G9" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="H9" s="3">
         <v>46266</v>
@@ -6018,10 +5966,10 @@
         <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="G14" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="H14" s="3">
         <v>46478</v>
@@ -6041,10 +5989,10 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="G15" t="s">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="H15" s="3">
         <v>46508</v>
@@ -6090,7 +6038,7 @@
         <v>162</v>
       </c>
       <c r="G17" t="s">
-        <v>556</v>
+        <v>550</v>
       </c>
       <c r="H17" s="3">
         <v>46631</v>
@@ -6136,7 +6084,7 @@
         <v>59</v>
       </c>
       <c r="G19" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="H19" s="3">
         <v>46661</v>
@@ -6159,7 +6107,7 @@
         <v>134</v>
       </c>
       <c r="G20" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="H20" s="3">
         <v>46661</v>
@@ -6251,7 +6199,7 @@
         <v>19</v>
       </c>
       <c r="G24" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H24" s="3">
         <v>46844</v>
@@ -6274,7 +6222,7 @@
         <v>44</v>
       </c>
       <c r="G25" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="H25" s="3">
         <v>46844</v>
@@ -6297,7 +6245,7 @@
         <v>59</v>
       </c>
       <c r="G26" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="H26" s="3">
         <v>46844</v>
@@ -6366,7 +6314,7 @@
         <v>470</v>
       </c>
       <c r="G29" t="s">
-        <v>562</v>
+        <v>556</v>
       </c>
       <c r="H29" s="3">
         <v>46905</v>
@@ -6389,7 +6337,7 @@
         <v>470</v>
       </c>
       <c r="G30" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="H30" s="3">
         <v>46905</v>
@@ -6412,7 +6360,7 @@
         <v>19</v>
       </c>
       <c r="G31" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H31" s="3">
         <v>46997</v>
@@ -6481,7 +6429,7 @@
         <v>13</v>
       </c>
       <c r="G34" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="H34" s="3">
         <v>47027</v>
@@ -6527,7 +6475,7 @@
         <v>162</v>
       </c>
       <c r="G36" t="s">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="H36" s="3">
         <v>47058</v>
@@ -6573,7 +6521,7 @@
         <v>59</v>
       </c>
       <c r="G38" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="H38" s="3">
         <v>47088</v>
@@ -6596,7 +6544,7 @@
         <v>59</v>
       </c>
       <c r="G39" t="s">
-        <v>565</v>
+        <v>559</v>
       </c>
       <c r="H39" s="3">
         <v>47150</v>
@@ -6619,7 +6567,7 @@
         <v>44</v>
       </c>
       <c r="G40" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="H40" s="3">
         <v>47178</v>
@@ -6685,10 +6633,10 @@
         <v>29</v>
       </c>
       <c r="F43" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="G43" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
       <c r="H43" s="3">
         <v>47270</v>
@@ -6754,10 +6702,10 @@
         <v>18</v>
       </c>
       <c r="F46" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="G46" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="H46" s="3">
         <v>47423</v>
@@ -6849,7 +6797,7 @@
         <v>134</v>
       </c>
       <c r="G50" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="H50" s="3">
         <v>47515</v>
@@ -6941,7 +6889,7 @@
         <v>480</v>
       </c>
       <c r="G54" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="H54" s="3">
         <v>47727</v>
@@ -6987,7 +6935,7 @@
         <v>44</v>
       </c>
       <c r="G56" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="H56" s="3">
         <v>47939</v>
@@ -7010,7 +6958,7 @@
         <v>59</v>
       </c>
       <c r="G57" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="H57" s="3">
         <v>47939</v>
@@ -7033,7 +6981,7 @@
         <v>134</v>
       </c>
       <c r="G58" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="H58" s="3">
         <v>47939</v>
@@ -7056,7 +7004,7 @@
         <v>19</v>
       </c>
       <c r="G59" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="H59" s="3">
         <v>47969</v>
@@ -7102,7 +7050,7 @@
         <v>134</v>
       </c>
       <c r="G61" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="H61" s="3">
         <v>47969</v>
@@ -7125,7 +7073,7 @@
         <v>13</v>
       </c>
       <c r="G62" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="H62" s="3">
         <v>48000</v>
@@ -7171,7 +7119,7 @@
         <v>13</v>
       </c>
       <c r="G64" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="H64" s="3">
         <v>48092</v>
@@ -7240,7 +7188,7 @@
         <v>19</v>
       </c>
       <c r="G67" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="H67" s="3">
         <v>48122</v>
@@ -7263,7 +7211,7 @@
         <v>19</v>
       </c>
       <c r="G68" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H68" s="3">
         <v>48305</v>
@@ -7286,7 +7234,7 @@
         <v>19</v>
       </c>
       <c r="G69" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H69" s="3">
         <v>48305</v>
@@ -7306,10 +7254,10 @@
         <v>29</v>
       </c>
       <c r="F70" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="G70" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="H70" s="3">
         <v>48305</v>
@@ -7329,10 +7277,10 @@
         <v>18</v>
       </c>
       <c r="F71" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="G71" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="H71" s="3">
         <v>48305</v>
@@ -7352,10 +7300,10 @@
         <v>29</v>
       </c>
       <c r="F72" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
       <c r="G72" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="H72" s="3">
         <v>48305</v>
@@ -7378,7 +7326,7 @@
         <v>19</v>
       </c>
       <c r="G73" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="H73" s="3">
         <v>48335</v>
@@ -7401,7 +7349,7 @@
         <v>134</v>
       </c>
       <c r="G74" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="H74" s="3">
         <v>48335</v>
@@ -7424,7 +7372,7 @@
         <v>13</v>
       </c>
       <c r="G75" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="H75" s="3">
         <v>48366</v>
@@ -7447,7 +7395,7 @@
         <v>134</v>
       </c>
       <c r="G76" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="H76" s="3">
         <v>48366</v>
@@ -7516,7 +7464,7 @@
         <v>134</v>
       </c>
       <c r="G79" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="H79" s="3">
         <v>48488</v>
@@ -7585,7 +7533,7 @@
         <v>44</v>
       </c>
       <c r="G82" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="H82" s="3">
         <v>48488</v>
@@ -7631,7 +7579,7 @@
         <v>59</v>
       </c>
       <c r="G84" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="H84" s="3">
         <v>48639</v>
@@ -7651,10 +7599,10 @@
         <v>18</v>
       </c>
       <c r="F85" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="G85" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="H85" s="3">
         <v>48670</v>
@@ -7677,7 +7625,7 @@
         <v>59</v>
       </c>
       <c r="G86" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="H86" s="3">
         <v>48700</v>
@@ -7700,7 +7648,7 @@
         <v>354</v>
       </c>
       <c r="G87" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="H87" s="3">
         <v>48700</v>
@@ -7723,7 +7671,7 @@
         <v>13</v>
       </c>
       <c r="G88" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="H88" s="3">
         <v>48700</v>
@@ -7769,7 +7717,7 @@
         <v>134</v>
       </c>
       <c r="G90" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="H90" s="3">
         <v>48731</v>
@@ -7861,7 +7809,7 @@
         <v>13</v>
       </c>
       <c r="G94" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="H94" s="3">
         <v>48823</v>
@@ -7953,7 +7901,7 @@
         <v>19</v>
       </c>
       <c r="G98" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="H98" s="3">
         <v>48884</v>
@@ -7976,7 +7924,7 @@
         <v>485</v>
       </c>
       <c r="G99" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="H99" s="3">
         <v>48884</v>
@@ -7996,10 +7944,10 @@
         <v>18</v>
       </c>
       <c r="F100" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="G100" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="H100" s="3">
         <v>48945</v>
@@ -8022,7 +7970,7 @@
         <v>134</v>
       </c>
       <c r="G101" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="H101" s="3">
         <v>48945</v>
@@ -8045,7 +7993,7 @@
         <v>342</v>
       </c>
       <c r="G102" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="H102" s="3">
         <v>48976</v>
@@ -8091,7 +8039,7 @@
         <v>13</v>
       </c>
       <c r="G104" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="H104" s="3">
         <v>49004</v>
@@ -8137,7 +8085,7 @@
         <v>134</v>
       </c>
       <c r="G106" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="H106" s="3">
         <v>49035</v>
@@ -8206,7 +8154,7 @@
         <v>13</v>
       </c>
       <c r="G109" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="H109" s="3">
         <v>49065</v>
@@ -8298,7 +8246,7 @@
         <v>59</v>
       </c>
       <c r="G113" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="H113" s="3">
         <v>49188</v>
@@ -8344,7 +8292,7 @@
         <v>19</v>
       </c>
       <c r="G115" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H115" s="3">
         <v>49188</v>
@@ -8367,7 +8315,7 @@
         <v>134</v>
       </c>
       <c r="G116" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="H116" s="3">
         <v>49218</v>
@@ -8390,7 +8338,7 @@
         <v>342</v>
       </c>
       <c r="G117" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="H117" s="3">
         <v>49218</v>
@@ -8413,7 +8361,7 @@
         <v>134</v>
       </c>
       <c r="G118" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="H118" s="3">
         <v>49249</v>
@@ -8490,22 +8438,22 @@
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
       <c r="C122" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="D122" t="s">
-        <v>593</v>
+        <v>587</v>
       </c>
       <c r="E122" t="s">
         <v>18</v>
       </c>
       <c r="F122" t="s">
-        <v>524</v>
+        <v>588</v>
       </c>
       <c r="G122" t="s">
-        <v>525</v>
+        <v>589</v>
       </c>
       <c r="H122" s="3">
         <v>49400</v>
@@ -8574,7 +8522,7 @@
         <v>13</v>
       </c>
       <c r="G125" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="H125" s="3">
         <v>49491</v>
@@ -8619,47 +8567,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>